<commit_message>
feat(v3): Task 7 — retitle all 22 published advertisements in manifest and tracker
- "With best compliments from [Company]" applied via targeted manifest line edits and a snapshot-first tracker write
- Added shared tracker-io.mjs; excluded advertisements untouched
- Tests: 1 integration (idempotent, 22 titles, tracker isolation)
- Security: semgrep clean, npm audit unchanged

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uai2kBaFAYKD1QqLxvNUw7
</commit_message>
<xml_diff>
--- a/04_MAGAZINE_WORKING/BECAA_2026_Content_Tracker.xlsx
+++ b/04_MAGAZINE_WORKING/BECAA_2026_Content_Tracker.xlsx
@@ -1357,7 +1357,7 @@
         <v>ADV-001</v>
       </c>
       <c r="B21" t="str">
-        <v>Skylark Advertisement</v>
+        <v>With best compliments from Skylark</v>
       </c>
       <c r="C21" t="str">
         <v>Advertisement</v>
@@ -1402,7 +1402,7 @@
         <v>Yes</v>
       </c>
       <c r="Q21" t="str">
-        <v>Preferred artwork: 1 Skylark.png. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 1 Skylark.png. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="22" ht="22.05" customHeight="1">
@@ -1410,7 +1410,7 @@
         <v>ADV-002</v>
       </c>
       <c r="B22" t="str">
-        <v>PNB Housing Advertisement</v>
+        <v>With best compliments from PNB Housing</v>
       </c>
       <c r="C22" t="str">
         <v>Advertisement</v>
@@ -1455,7 +1455,7 @@
         <v>Yes</v>
       </c>
       <c r="Q22" t="str">
-        <v>Preferred artwork: 2 d PNB FD Magazine AD_A4-01.pdf. Selected full-page A4 file explicitly named Magazine AD; other PNB files are alternate designs/logo.</v>
+        <v>Preferred artwork: 2 d PNB FD Magazine AD_A4-01.pdf. Selected full-page A4 file explicitly named Magazine AD; other PNB files are alternate designs/logo. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="23" ht="22.05" customHeight="1">
@@ -1463,7 +1463,7 @@
         <v>ADV-003</v>
       </c>
       <c r="B23" t="str">
-        <v>Vistaar Finance Advertisement</v>
+        <v>With best compliments from Vistaar Finance</v>
       </c>
       <c r="C23" t="str">
         <v>Advertisement</v>
@@ -1508,7 +1508,7 @@
         <v>Yes</v>
       </c>
       <c r="Q23" t="str">
-        <v>Preferred artwork: 3 Vistaar Finance.jpg. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 3 Vistaar Finance.jpg. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="24" ht="22.05" customHeight="1">
@@ -1516,7 +1516,7 @@
         <v>ADV-004</v>
       </c>
       <c r="B24" t="str">
-        <v>Gainwell Technologies Advertisement</v>
+        <v>With best compliments from Gainwell Technologies</v>
       </c>
       <c r="C24" t="str">
         <v>Advertisement</v>
@@ -1561,7 +1561,7 @@
         <v>Yes</v>
       </c>
       <c r="Q24" t="str">
-        <v>Preferred artwork: 4 Gainwell Technologies.jpg. Selected primary company artwork; CAT image is supplemental alternate artwork.</v>
+        <v>Preferred artwork: 4 Gainwell Technologies.jpg. Selected primary company artwork; CAT image is supplemental alternate artwork. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="25" ht="22.05" customHeight="1">
@@ -1569,7 +1569,7 @@
         <v>ADV-005</v>
       </c>
       <c r="B25" t="str">
-        <v>Tata Capital Ltd. Retail Finance Advertisement</v>
+        <v>With best compliments from Tata Capital Ltd. (Retail Finance)</v>
       </c>
       <c r="C25" t="str">
         <v>Advertisement</v>
@@ -1614,7 +1614,7 @@
         <v>Yes</v>
       </c>
       <c r="Q25" t="str">
-        <v>Preferred artwork: 5a Tata Capital ltd. (Retail Finance).jpg. Selected full-page retail-finance artwork; base file is logo-only.</v>
+        <v>Preferred artwork: 5a Tata Capital ltd. (Retail Finance).jpg. Selected full-page retail-finance artwork; base file is logo-only. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="26" ht="22.05" customHeight="1">
@@ -1622,7 +1622,7 @@
         <v>ADV-006</v>
       </c>
       <c r="B26" t="str">
-        <v>Tata Capital Housing Finance Ltd. Advertisement</v>
+        <v>With best compliments from Tata Capital Housing Finance Ltd.</v>
       </c>
       <c r="C26" t="str">
         <v>Advertisement</v>
@@ -1667,7 +1667,7 @@
         <v>Yes</v>
       </c>
       <c r="Q26" t="str">
-        <v>Preferred artwork: 6 d tata capital.pdf. Selected full portrait PDF advertisement; JPG files are alternate banners/placements.</v>
+        <v>Preferred artwork: 6 d tata capital.pdf. Selected full portrait PDF advertisement; JPG files are alternate banners/placements. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="27" ht="22.05" customHeight="1">
@@ -1675,7 +1675,7 @@
         <v>ADV-007</v>
       </c>
       <c r="B27" t="str">
-        <v>OnShore Construction Pvt Ltd Advertisement</v>
+        <v>With best compliments from OnShore Construction Pvt Ltd</v>
       </c>
       <c r="C27" t="str">
         <v>Advertisement</v>
@@ -1720,7 +1720,7 @@
         <v>Yes</v>
       </c>
       <c r="Q27" t="str">
-        <v>Preferred artwork: 7 OnShore Construction Pvt Ltd .png. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 7 OnShore Construction Pvt Ltd .png. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="28" ht="22.05" customHeight="1">
@@ -1728,7 +1728,7 @@
         <v>ADV-008</v>
       </c>
       <c r="B28" t="str">
-        <v>Roofs &amp; Ceilings Advertisement</v>
+        <v>With best compliments from Roofs &amp; Ceilings</v>
       </c>
       <c r="C28" t="str">
         <v>Advertisement</v>
@@ -1773,7 +1773,7 @@
         <v>Yes</v>
       </c>
       <c r="Q28" t="str">
-        <v>Preferred artwork: 8 Roofs &amp; Ceilings.png. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 8 Roofs &amp; Ceilings.png. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="29" ht="22.05" customHeight="1">
@@ -1834,7 +1834,7 @@
         <v>ADV-010</v>
       </c>
       <c r="B30" t="str">
-        <v>Indus Grand Advertisement</v>
+        <v>With best compliments from Indus Grand</v>
       </c>
       <c r="C30" t="str">
         <v>Advertisement</v>
@@ -1879,7 +1879,7 @@
         <v>Yes</v>
       </c>
       <c r="Q30" t="str">
-        <v>Preferred artwork: 10 Indus Grand.jpeg. Selected full advertisement; 10a is logo-only.</v>
+        <v>Preferred artwork: 10 Indus Grand.jpeg. Selected full advertisement; 10a is logo-only. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="31" ht="22.05" customHeight="1">
@@ -1887,7 +1887,7 @@
         <v>ADV-011</v>
       </c>
       <c r="B31" t="str">
-        <v>Axelon Advertisement</v>
+        <v>With best compliments from Axelon</v>
       </c>
       <c r="C31" t="str">
         <v>Advertisement</v>
@@ -1932,7 +1932,7 @@
         <v>Yes</v>
       </c>
       <c r="Q31" t="str">
-        <v>Preferred artwork: 11 Axelon.jpg. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 11 Axelon.jpg. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="32" ht="22.05" customHeight="1">
@@ -1940,7 +1940,7 @@
         <v>ADV-012</v>
       </c>
       <c r="B32" t="str">
-        <v>Aarvi Encon Advertisement</v>
+        <v>With best compliments from Aarvi Encon</v>
       </c>
       <c r="C32" t="str">
         <v>Advertisement</v>
@@ -1985,7 +1985,7 @@
         <v>Yes</v>
       </c>
       <c r="Q32" t="str">
-        <v>Preferred artwork: 12 arvi enercon.jpeg. Exact tracker file exists; artwork and sponsor workbook confirm Aarvi Encon despite filename spelling.</v>
+        <v>Preferred artwork: 12 arvi enercon.jpeg. Exact tracker file exists; artwork and sponsor workbook confirm Aarvi Encon despite filename spelling. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="33" ht="22.05" customHeight="1">
@@ -1993,7 +1993,7 @@
         <v>ADV-013</v>
       </c>
       <c r="B33" t="str">
-        <v>Anand Rathi Advertisement</v>
+        <v>With best compliments from Anand Rathi</v>
       </c>
       <c r="C33" t="str">
         <v>Advertisement</v>
@@ -2038,7 +2038,7 @@
         <v>Yes</v>
       </c>
       <c r="Q33" t="str">
-        <v>Preferred artwork: 13a Anand Rathi.jpeg. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 13a Anand Rathi.jpeg. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="34" ht="22.05" customHeight="1">
@@ -2046,7 +2046,7 @@
         <v>ADV-014</v>
       </c>
       <c r="B34" t="str">
-        <v>Future Netwings Solutions Advertisement</v>
+        <v>With best compliments from Future Netwings Solutions</v>
       </c>
       <c r="C34" t="str">
         <v>Advertisement</v>
@@ -2091,7 +2091,7 @@
         <v>Yes</v>
       </c>
       <c r="Q34" t="str">
-        <v>Preferred artwork: 14 a future netwings.pdf. Selected full-page PDF; PNG files are logo/raster derivative alternatives.</v>
+        <v>Preferred artwork: 14 a future netwings.pdf. Selected full-page PDF; PNG files are logo/raster derivative alternatives. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="35" ht="22.05" customHeight="1">
@@ -2099,7 +2099,7 @@
         <v>ADV-015</v>
       </c>
       <c r="B35" t="str">
-        <v>Swaraj Shoes Advertisement</v>
+        <v>With best compliments from Swaraj Shoes</v>
       </c>
       <c r="C35" t="str">
         <v>Advertisement</v>
@@ -2144,7 +2144,7 @@
         <v>Yes</v>
       </c>
       <c r="Q35" t="str">
-        <v>Preferred artwork: 15 Swaraj Shoes.jpeg. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 15 Swaraj Shoes.jpeg. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="36" ht="22.05" customHeight="1">
@@ -2205,7 +2205,7 @@
         <v>ADV-017</v>
       </c>
       <c r="B37" t="str">
-        <v>UREDCONNECT Advertisement</v>
+        <v>With best compliments from UREDCONNECT</v>
       </c>
       <c r="C37" t="str">
         <v>Advertisement</v>
@@ -2250,7 +2250,7 @@
         <v>Yes</v>
       </c>
       <c r="Q37" t="str">
-        <v>Preferred artwork: 17 UREDCONNECT.jpeg. Selected primary numbered advertisement; 17a is an alternate design.</v>
+        <v>Preferred artwork: 17 UREDCONNECT.jpeg. Selected primary numbered advertisement; 17a is an alternate design. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="38" ht="22.05" customHeight="1">
@@ -2258,7 +2258,7 @@
         <v>ADV-018</v>
       </c>
       <c r="B38" t="str">
-        <v>Eframe Advertisement</v>
+        <v>With best compliments from Eframe</v>
       </c>
       <c r="C38" t="str">
         <v>Advertisement</v>
@@ -2303,7 +2303,7 @@
         <v>Yes</v>
       </c>
       <c r="Q38" t="str">
-        <v>Preferred artwork: 18 Eframe.jpeg. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 18 Eframe.jpeg. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="39" ht="22.05" customHeight="1">
@@ -2311,7 +2311,7 @@
         <v>ADV-019</v>
       </c>
       <c r="B39" t="str">
-        <v>Network Techlabs Advertisement</v>
+        <v>With best compliments from Network Techlabs</v>
       </c>
       <c r="C39" t="str">
         <v>Advertisement</v>
@@ -2356,7 +2356,7 @@
         <v>Yes</v>
       </c>
       <c r="Q39" t="str">
-        <v>Preferred artwork: 19 Network Techlabs.png. Selected primary numbered artwork; 19A is an alternate banner.</v>
+        <v>Preferred artwork: 19 Network Techlabs.png. Selected primary numbered artwork; 19A is an alternate banner. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="40" ht="22.05" customHeight="1">
@@ -2364,7 +2364,7 @@
         <v>ADV-020</v>
       </c>
       <c r="B40" t="str">
-        <v>Schnelltech Global Advertisement</v>
+        <v>With best compliments from Schnelltech Global</v>
       </c>
       <c r="C40" t="str">
         <v>Advertisement</v>
@@ -2409,7 +2409,7 @@
         <v>Yes</v>
       </c>
       <c r="Q40" t="str">
-        <v>Preferred artwork: 20 b Schnelltech Global.pdf. Selected full magazine PDF; base file is logo-only and 20a is a raster derivative.</v>
+        <v>Preferred artwork: 20 b Schnelltech Global.pdf. Selected full magazine PDF; base file is logo-only and 20a is a raster derivative. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="41" ht="22.05" customHeight="1">
@@ -2417,7 +2417,7 @@
         <v>ADV-021</v>
       </c>
       <c r="B41" t="str">
-        <v>Bhavik Advertisement</v>
+        <v>With best compliments from Bhavik</v>
       </c>
       <c r="C41" t="str">
         <v>Advertisement</v>
@@ -2462,7 +2462,7 @@
         <v>Yes</v>
       </c>
       <c r="Q41" t="str">
-        <v>Preferred artwork: 21 Bhavik.jpeg. Company name corrected to Bhavik from the name displayed in the approved artwork, per user authorization.</v>
+        <v>Preferred artwork: 21 Bhavik.jpeg. Company name corrected to Bhavik from the name displayed in the approved artwork, per user authorization. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="42" ht="22.05" customHeight="1">
@@ -2470,7 +2470,7 @@
         <v>ADV-022</v>
       </c>
       <c r="B42" t="str">
-        <v>Pratap Caterer Advertisement</v>
+        <v>With best compliments from Pratap Caterer</v>
       </c>
       <c r="C42" t="str">
         <v>Advertisement</v>
@@ -2515,7 +2515,7 @@
         <v>Yes</v>
       </c>
       <c r="Q42" t="str">
-        <v>Preferred artwork: 22 pratap caterer.png. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 22 pratap caterer.png. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="43" ht="22.05" customHeight="1">
@@ -2523,7 +2523,7 @@
         <v>ADV-023</v>
       </c>
       <c r="B43" t="str">
-        <v>Clover Blakefield Reality LLP Advertisement</v>
+        <v>With best compliments from Clover Blakefield Reality LLP</v>
       </c>
       <c r="C43" t="str">
         <v>Advertisement</v>
@@ -2568,7 +2568,7 @@
         <v>Yes</v>
       </c>
       <c r="Q43" t="str">
-        <v>Preferred artwork: 23 Clover Blakefield Reality LLP.png. Exact available artwork matched to tracker row.</v>
+        <v>Preferred artwork: 23 Clover Blakefield Reality LLP.png. Exact available artwork matched to tracker row. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="44" ht="22.05" customHeight="1">
@@ -2682,7 +2682,7 @@
         <v>ADV-026</v>
       </c>
       <c r="B46" t="str">
-        <v>CETEST Advertisement</v>
+        <v>With best compliments from CETEST</v>
       </c>
       <c r="C46" t="str">
         <v>Advertisement</v>
@@ -2727,7 +2727,7 @@
         <v>Yes</v>
       </c>
       <c r="Q46" t="str">
-        <v>Explicitly approved for 2026 review publication. Render slide 1 from the original PPTX with LibreOffice Impress PDF export, then rasterize at 300 DPI; preserve original PPTX untouched.</v>
+        <v>Explicitly approved for 2026 review publication. Render slide 1 from the original PPTX with LibreOffice Impress PDF export, then rasterize at 300 DPI; preserve original PPTX untouched. Sprint v3 (2026-09-14): public display title changed to "With best compliments from [Company]" per sprints/v3/PRD.md §4.3; artwork, source file and normalized files unchanged.</v>
       </c>
     </row>
     <row r="47" ht="22.05" customHeight="1">

</xml_diff>

<commit_message>
feat(v3): Task 8 — record Item 18 revision and approve Item 24 in the tracker
- Pure applyTrackerFieldUpdates() + snapshot-first apply script (rows 18 and 24 only)
- Tests: 3 unit groups, 1 idempotent integration
- Security: semgrep clean, npm audit unchanged
- Note: tracker:validate's stale Item-24 rule now fails by design until Task 9

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uai2kBaFAYKD1QqLxvNUw7
</commit_message>
<xml_diff>
--- a/04_MAGAZINE_WORKING/BECAA_2026_Content_Tracker.xlsx
+++ b/04_MAGAZINE_WORKING/BECAA_2026_Content_Tracker.xlsx
@@ -1296,7 +1296,7 @@
         <v>Yes</v>
       </c>
       <c r="Q19" t="str">
-        <v/>
+        <v>Sprint v3: revised source received 2026-09-14 (SHA-256 ed3fd766…) replaces the 01.08.2026 version (SHA-256 df446f44…), preserved in 04_MAGAZINE_WORKING/SUPERSEDED_SOURCES/2026-09-14/ and git history.</v>
       </c>
     </row>
     <row r="20" ht="22.05" customHeight="1">
@@ -3053,7 +3053,7 @@
         <v>24</v>
       </c>
       <c r="B53" t="str">
-        <v>Siddhartha Mukhopadhyay story</v>
+        <v>প্যাঁড়া (Siddhartha Mukhopadhyay story)</v>
       </c>
       <c r="C53" t="str">
         <v>Story</v>
@@ -3071,13 +3071,13 @@
         <v>Siddhartha Mukhopadhyay story.docx</v>
       </c>
       <c r="H53" t="str">
-        <v/>
+        <v>14.09.2026</v>
       </c>
       <c r="I53" t="str">
-        <v>Pending</v>
+        <v>Print and web</v>
       </c>
       <c r="J53" t="str">
-        <v>Excluded – Content and permission pending</v>
+        <v>Approved</v>
       </c>
       <c r="K53" t="str">
         <v>College Memories</v>
@@ -3086,7 +3086,7 @@
         <v/>
       </c>
       <c r="M53" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="N53" t="str">
         <v/>
@@ -3095,10 +3095,10 @@
         <v/>
       </c>
       <c r="P53" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="Q53" t="str">
-        <v>Sprint v2: source docx contains only placeholder text ("Story upcoming.") and Permission is still Pending. Excluded until real content and permission are both received. See sprints/v2/MATERIAL_CHANGE_REGISTER.md.</v>
+        <v>Sprint v2: source docx contains only placeholder text ("Story upcoming.") and Permission is still Pending. Excluded until real content and permission are both received. See sprints/v2/MATERIAL_CHANGE_REGISTER.md. Sprint v3: real content received and approval confirmed 2026-09-14; published as ART-012.</v>
       </c>
     </row>
     <row r="54" ht="22.05" customHeight="1"/>

</xml_diff>